<commit_message>
Admin shabloni (13 ustun) va safdan chiqarish / akademik ta'til buyrug'i
- QABUL - 2026 va Baza administratori: administratorning "Qabul uchun
  shablon.xlsx" fayli bilan aynan bir xil — bitta "Лист1" sahifa, 3-qatorda
  sarlavha, 13 ustun (ruscha yo'q), shablondagi kenglik va shriftlar
  (portal, generate_qabul_shablon.py va xizmatdagi admin fayli)
- Talaba safdan chiqarilganda yoki akademik ta'tilga o'tkazilganda buyruq
  raqami va sanasi so'raladi (BuyruqModal, tahrirlash formasi); Excelning
  26–27-ustunlarida saqlanadi, students.json ga buyruq/buyruq_sana
- Xizmat: do_GET ichidagi mahalliy "import urllib.request" rol fayllarini
  eksport qilish va Telegramga yuborishni UnboundLocalError bilan buzardi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hisobotlar/qabul/guruhlar/QABUL - 2026 (26-01).xlsx
+++ b/hisobotlar/qabul/guruhlar/QABUL - 2026 (26-01).xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,37 +27,15 @@
     </font>
     <font>
       <name val="Times New Roman"/>
-      <b val="1"/>
-      <color rgb="001E3A8A"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <i val="1"/>
-      <color rgb="00555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8EEF5"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -86,22 +64,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,954 +435,864 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A3:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4.5" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="17.5" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="16.5" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="3.14" customWidth="1" min="1" max="1"/>
+    <col width="34.43" customWidth="1" min="2" max="2"/>
+    <col width="17.29" customWidth="1" min="3" max="3"/>
+    <col width="13.43" customWidth="1" min="4" max="4"/>
+    <col width="17.86" customWidth="1" min="5" max="5"/>
+    <col width="22.57" customWidth="1" min="6" max="6"/>
+    <col width="21.71" customWidth="1" min="7" max="7"/>
+    <col width="17.71" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="26.29" customWidth="1" min="10" max="10"/>
+    <col width="13.86" customWidth="1" min="11" max="11"/>
+    <col width="16.43" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Guruh 26-01 (14 nafar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Namuna: Saydalimov Anvarjon Sarvarjon o`g`li | 517******0016 | AC1686958 | 990201527 | Qashqadaryo, Qarshi | 4-mittituman 21/23 | Qarshi shahar 1-maktab | Qarshi City School No. 1 | Школа №1 города Карши | Maktab | AA1775603 | 2008-2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="63" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="47.25" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>F.I.O</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>JSHSHIR</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Pasport seriya raqami</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Tel raqam(pastdagi shablondagidek kiritilsin)</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>2-Tel raqam(pastdagi shablondagidek kiritilsin)</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>Yashash viloyat+tumani</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>UY manzili</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>Avval o`qigan muassasa nomi(Uzbek tilida)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>Avval o`qigan muassasa nomi(Ingliz tilida)</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Avval o`qigan muassasa nomi(Rus tilida)</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>Maktab, kollej va HK</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>Avval olgan diplom seriya+raqami</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr">
         <is>
           <t>Boshlagan va tugatgan yili</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="4" t="n">
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Abdijalolova Dilnura Yusufjon qizi</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>62703085680021</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>AE3226696</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="2" t="n">
         <v>996810119</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="2" t="n">
         <v>978550581</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 28-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 28, Kitob District</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №28 Китабского района</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>UM 03728883</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="n">
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Abdurahmonova Parvinabonu Alisher qizi</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>61402095680050</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>AE2261219</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="2" t="n">
         <v>885888187</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="2" t="n">
         <v>902433774</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 4-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 4, Kitob District</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №4 Китабского района</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>UM 03727987</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="4" t="n">
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Arzikulova Amina Salohiddin qizi</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>61204085590053</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>AD6876141</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="2" t="n">
         <v>953672602</v>
       </c>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 15, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №15 Шахрисабзского района</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>UM 03752576</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="4" t="n">
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Azamatova Charos Abdiaziz qizi</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>61102085590018</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>AE1520971</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 39-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 39, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №39 Шахрисабзского района</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>UM 03754638</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="4" t="n">
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Hazratova Farzona Toshkand qizi</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>62305075590039</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>AD5641030</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="2" t="n">
         <v>914606562</v>
       </c>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 26-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 26, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №26 Шахрисабзского района</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>UM 02167009</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>2013-2024</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="n">
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Ibodullayeva Asilzoda Latif qizi</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>62610085590024</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>AD9929006</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="2" t="n">
         <v>973873803</v>
       </c>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 14-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 14, Shahrisabz City</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №14 города Шахрисабз</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>UM 03752500</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="4" t="n">
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Majidova Namuna Shunqor qizi</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>61106005680025</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>AB6959094</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="2" t="n">
         <v>943387727</v>
       </c>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Kitob qishloq xo'jalik kasb-hunar kolleji</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Kitob Agricultural Vocational College</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>Китабский сельскохозяйственный профессиональный колледж</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Kollej</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>K 5487890</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>2016-2019</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="n">
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Meliyeva Umida Shavkat qizi</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>42603932560110</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>AB9495274</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz Tibbiyot Kolleji</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz Medical College</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>Шахрисабзский медицинский колледж</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Kollej</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>K 2411482</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>2009-2012</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="4" t="n">
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Murodullayev Azizbek Odiljon o'g'li</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>52011075590034</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>AD6281528</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="2" t="n">
         <v>919490180</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="F12" s="2" t="n">
         <v>877511981</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 14, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №14 Шахрисабзского района</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>UM 03296171</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>2014-2025</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="4" t="n">
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Numonova Jasmina Baxodir qizi</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>61705085590020</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>AE1748671</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="2" t="n">
         <v>509071311</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" s="2" t="n">
         <v>500331311</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 7-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 7, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №7 Шахрисабзского района</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>UM 03751929</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="4" t="n">
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Ravshanova Ruhshona Radju qizi</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>60204095680082</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>AE6085379</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="2" t="n">
         <v>908788108</v>
       </c>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 1-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 1, Kitob District</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №1 Китабского района</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>UM 03727735</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="4" t="n">
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Turayeva Dilsuz Oybek qizi</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>61205095590053</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>AE5053541</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="2" t="n">
         <v>936031585</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" s="2" t="n">
         <v>882651585</v>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 2-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 2, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №2 Шахрисабзского района</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>UM 03751635</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="4" t="n">
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Turg'unova Jasmina Turg'un qizi</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>62802085590087</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>AE6171425</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="2" t="n">
         <v>910707501</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F16" s="2" t="n">
         <v>908698209</v>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 2-son politexnikumi</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Polytechnic College No. 2, Shahrisabz City</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>Политехникум №2 города Шахрисабз</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Texnikum</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>PT 0339231</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>2023-2026</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="n">
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Ziyodullayeva Jasmina Alisher qizi</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>61206075590076</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>AD9812146</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="2" t="n">
         <v>912240018</v>
       </c>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 14, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>Общеобразовательная школа №14 Шахрисабзского района</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>UM 03296188</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>2014-2025</t>
         </is>

</xml_diff>

<commit_message>
QABUL - 2026 va Baza administratori: Guruhi ustuni qo'shildi (A: №, B: Guruhi, C: F.I.O)
</commit_message>
<xml_diff>
--- a/hisobotlar/qabul/guruhlar/QABUL - 2026 (26-01).xlsx
+++ b/hisobotlar/qabul/guruhlar/QABUL - 2026 (26-01).xlsx
@@ -435,22 +435,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:M17"/>
+  <dimension ref="A3:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.14" customWidth="1" min="1" max="1"/>
-    <col width="34.43" customWidth="1" min="2" max="2"/>
-    <col width="17.29" customWidth="1" min="3" max="3"/>
-    <col width="13.43" customWidth="1" min="4" max="4"/>
-    <col width="17.86" customWidth="1" min="5" max="5"/>
-    <col width="22.57" customWidth="1" min="6" max="6"/>
-    <col width="21.71" customWidth="1" min="7" max="7"/>
-    <col width="17.71" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="26.29" customWidth="1" min="10" max="10"/>
-    <col width="13.86" customWidth="1" min="11" max="11"/>
-    <col width="16.43" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="34.43" customWidth="1" min="3" max="3"/>
+    <col width="17.29" customWidth="1" min="4" max="4"/>
+    <col width="13.43" customWidth="1" min="5" max="5"/>
+    <col width="17.86" customWidth="1" min="6" max="6"/>
+    <col width="22.57" customWidth="1" min="7" max="7"/>
+    <col width="21.71" customWidth="1" min="8" max="8"/>
+    <col width="17.71" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="26.29" customWidth="1" min="11" max="11"/>
+    <col width="13.86" customWidth="1" min="12" max="12"/>
+    <col width="16.43" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="3" ht="47.25" customHeight="1">
@@ -461,60 +462,65 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
+          <t>Guruhi</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
           <t>F.I.O</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>JSHSHIR</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Pasport seriya raqami</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>Tel raqam(pastdagi shablondagidek kiritilsin)</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>2-Tel raqam(pastdagi shablondagidek kiritilsin)</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>Yashash viloyat+tumani</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>UY manzili</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>Avval o`qigan muassasa nomi(Uzbek tilida)</t>
         </is>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>Avval o`qigan muassasa nomi(Ingliz tilida)</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>Maktab, kollej va HK</t>
         </is>
       </c>
-      <c r="L3" s="1" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr">
         <is>
           <t>Avval olgan diplom seriya+raqami</t>
         </is>
       </c>
-      <c r="M3" s="1" t="inlineStr">
+      <c r="N3" s="1" t="inlineStr">
         <is>
           <t>Boshlagan va tugatgan yili</t>
         </is>
@@ -526,52 +532,57 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>Abdijalolova Dilnura Yusufjon qizi</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>62703085680021</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>AE3226696</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>996810119</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>978550581</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 28-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 28, Kitob District</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>UM 03728883</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
@@ -583,52 +594,57 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
           <t>Abdurahmonova Parvinabonu Alisher qizi</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>61402095680050</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>AE2261219</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>885888187</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>902433774</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 4-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 4, Kitob District</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>UM 03727987</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
@@ -640,50 +656,55 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>Arzikulova Amina Salohiddin qizi</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>61204085590053</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>AD6876141</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>953672602</v>
       </c>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 15, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>UM 03752576</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
@@ -695,48 +716,53 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>Azamatova Charos Abdiaziz qizi</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>61102085590018</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>AE1520971</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 39-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 39, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>UM 03754638</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
@@ -748,50 +774,55 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>Hazratova Farzona Toshkand qizi</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>62305075590039</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>AD5641030</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>914606562</v>
       </c>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 26-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 26, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>UM 02167009</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>2013-2024</t>
         </is>
@@ -803,50 +834,55 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>Ibodullayeva Asilzoda Latif qizi</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>62610085590024</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>AD9929006</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="F9" s="2" t="n">
         <v>973873803</v>
       </c>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 14-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 14, Shahrisabz City</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>UM 03752500</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
@@ -858,50 +894,55 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>Majidova Namuna Shunqor qizi</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>61106005680025</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>AB6959094</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="F10" s="2" t="n">
         <v>943387727</v>
       </c>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Kitob qishloq xo'jalik kasb-hunar kolleji</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Kitob Agricultural Vocational College</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Kollej</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>K 5487890</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>2016-2019</t>
         </is>
@@ -913,48 +954,53 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>Meliyeva Umida Shavkat qizi</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>42603932560110</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>AB9495274</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz Tibbiyot Kolleji</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz Medical College</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Kollej</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>K 2411482</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>2009-2012</t>
         </is>
@@ -966,52 +1012,57 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
           <t>Murodullayev Azizbek Odiljon o'g'li</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>52011075590034</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>AD6281528</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="F12" s="2" t="n">
         <v>919490180</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>877511981</v>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 14, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>UM 03296171</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>2014-2025</t>
         </is>
@@ -1023,52 +1074,57 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
           <t>Numonova Jasmina Baxodir qizi</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>61705085590020</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>AE1748671</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="F13" s="2" t="n">
         <v>509071311</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>500331311</v>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 7-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 7, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>UM 03751929</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
@@ -1080,50 +1136,55 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
           <t>Ravshanova Ruhshona Radju qizi</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>60204095680082</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>AE6085379</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="F14" s="2" t="n">
         <v>908788108</v>
       </c>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 1-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 1, Kitob District</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>UM 03727735</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
@@ -1135,52 +1196,57 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>Turayeva Dilsuz Oybek qizi</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>61205095590053</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>AE5053541</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="F15" s="2" t="n">
         <v>936031585</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>882651585</v>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 2-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 2, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>UM 03751635</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>
@@ -1192,52 +1258,57 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>Turg'unova Jasmina Turg'un qizi</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>62802085590087</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>AE6171425</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="F16" s="2" t="n">
         <v>910707501</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>908698209</v>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 2-son politexnikumi</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Polytechnic College No. 2, Shahrisabz City</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Texnikum</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>PT 0339231</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>2023-2026</t>
         </is>
@@ -1249,50 +1320,55 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
           <t>Ziyodullayeva Jasmina Alisher qizi</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>61206075590076</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>AD9812146</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="F17" s="2" t="n">
         <v>912240018</v>
       </c>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>General Secondary School No. 14, Shahrisabz District</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Maktab</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>UM 03296188</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>2014-2025</t>
         </is>

</xml_diff>